<commit_message>
purged resource pack and compressed textures
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\1.21.7\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50BAFFF3-6D03-45C0-98E8-DB7B0807BE1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{266EB93C-1AAC-46A7-8D5D-40C210FFFDCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Minecraft Version</t>
   </si>
@@ -73,6 +73,9 @@
   </si>
   <si>
     <t>Updated resource pack to work on 1.20 again</t>
+  </si>
+  <si>
+    <t>Fixed flowing water sound</t>
   </si>
 </sst>
 </file>
@@ -606,6 +609,11 @@
         <v>15</v>
       </c>
     </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
     <row r="21" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:A24">

</xml_diff>

<commit_message>
changed copper golem textures
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\1.21.7\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27BCA2B2-859A-4A41-865F-EFC4424CE5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C7D841A-24FB-4D9B-A4A1-B61F8633AA17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Minecraft Version</t>
   </si>
@@ -76,6 +76,9 @@
   </si>
   <si>
     <t>Added Copper Horse Armor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changed copper golem textures </t>
   </si>
 </sst>
 </file>
@@ -617,6 +620,11 @@
         <v>16</v>
       </c>
     </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
     <row r="21" ht="16.5" customHeight="1"/>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:A24">

</xml_diff>

<commit_message>
Added texture for the nautilus saddle
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\1.21.7\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9F81AB5-ED25-47CA-885A-5E795EE20607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{772D07B1-5289-468D-9742-6565CE250F55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Minecraft Version</t>
   </si>
@@ -93,6 +93,9 @@
   </si>
   <si>
     <t>Added nautilus armor item textures</t>
+  </si>
+  <si>
+    <t>Added texture for nautilus saddle</t>
   </si>
 </sst>
 </file>
@@ -559,8 +562,8 @@
         <v>14</v>
       </c>
       <c r="C2" s="6">
-        <f>SUM(2511,513,2025)</f>
-        <v>5049</v>
+        <f>SUM(2511,524,2025)</f>
+        <v>5060</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>8</v>
@@ -606,7 +609,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
@@ -615,7 +618,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
@@ -624,7 +627,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
@@ -633,28 +636,33 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>18</v>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:A10">
-    <sortCondition ref="A10"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:A13">
+    <sortCondition ref="A13"/>
   </sortState>
   <mergeCells count="4">
     <mergeCell ref="A3:B3"/>

</xml_diff>

<commit_message>
Added chest CEM (WIP)
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\1.21.7\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E33235CC-0C5A-4332-8868-AB32C7C66F31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7684896F-3B5F-497E-8D08-A67ACDDCDB32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Minecraft Version</t>
   </si>
@@ -69,6 +69,9 @@
   </si>
   <si>
     <t>Updated CEM (full fix for boats)</t>
+  </si>
+  <si>
+    <t>Added chest CEM (WIP)</t>
   </si>
 </sst>
 </file>
@@ -535,8 +538,8 @@
         <v>8</v>
       </c>
       <c r="C2" s="6">
-        <f>SUM(2511,539,2025)</f>
-        <v>5075</v>
+        <f>SUM(2511,544,2025)</f>
+        <v>5080</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>7</v>
@@ -572,6 +575,9 @@
       <c r="H4" s="8"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="E5" s="8"/>
       <c r="F5" s="8"/>
       <c r="G5" s="8"/>

</xml_diff>